<commit_message>
Fix Kobo GT HORECA metadata and PNG reports
</commit_message>
<xml_diff>
--- a/templates/KB_Market_Improvement_XLSForm_GT_HORECA.xlsx
+++ b/templates/KB_Market_Improvement_XLSForm_GT_HORECA.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="survey" sheetId="1" r:id="R044aa7db4e3046bd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="choices" sheetId="2" r:id="Ra4c39ed1d35e4b36"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="settings" sheetId="3" r:id="R464e73a2e02a4d0f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bot_Logic" sheetId="4" r:id="Rfb1a8fa6ff374df9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bot_Data_Map" sheetId="5" r:id="R2ac020d450774bb6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="survey" sheetId="1" r:id="R4f44dbec69b94b5e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="choices" sheetId="2" r:id="Raf5f1cd1db71408e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="settings" sheetId="3" r:id="R0d2a0057f05a49b2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bot_Logic" sheetId="4" r:id="Rc547f61ed6d1488c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bot_Data_Map" sheetId="5" r:id="Ra90132a7a14c451a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -754,9 +754,9 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Calibri"/>
-        <a:ea typeface="Calibri"/>
-        <a:cs typeface="Calibri"/>
+        <a:latin typeface="Calibri Light"/>
+        <a:ea typeface="Calibri Light"/>
+        <a:cs typeface="Calibri Light"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -942,7 +942,7 @@
         <x:v>Region</x:v>
       </x:c>
       <x:c r="D3" s="11" t="str">
-        <x:v>no</x:v>
+        <x:v>yes</x:v>
       </x:c>
       <x:c r="E3" s="11" t="str">
         <x:v>ជ្រើសរើស Region</x:v>
@@ -967,7 +967,7 @@
         <x:v>Dealer</x:v>
       </x:c>
       <x:c r="D4" s="11" t="str">
-        <x:v>no</x:v>
+        <x:v>yes</x:v>
       </x:c>
       <x:c r="E4" s="11" t="str">
         <x:v>Dealer list filters by Region</x:v>
@@ -1019,7 +1019,7 @@
         <x:v>Report Date</x:v>
       </x:c>
       <x:c r="D6" s="11" t="str">
-        <x:v>no</x:v>
+        <x:v>yes</x:v>
       </x:c>
       <x:c r="E6" s="11"/>
       <x:c r="F6" s="11"/>
@@ -1434,7 +1434,7 @@
       </x:c>
       <x:c r="G23" s="11"/>
       <x:c r="H23" s="11" t="str">
-        <x:v>${final_summary_report_type} = 'horeca'</x:v>
+        <x:v>string-length(normalize-space(${final_summary_report_type})) = 0 or ${final_summary_report_type} = 'horeca'</x:v>
       </x:c>
       <x:c r="I23" s="11"/>
       <x:c r="J23" s="11"/>
@@ -1582,7 +1582,7 @@
       </x:c>
       <x:c r="G29" s="11"/>
       <x:c r="H29" s="11" t="str">
-        <x:v>${final_summary_report_type} = 'horeca'</x:v>
+        <x:v>string-length(normalize-space(${final_summary_report_type})) = 0 or ${final_summary_report_type} = 'horeca'</x:v>
       </x:c>
       <x:c r="I29" s="11"/>
       <x:c r="J29" s="11"/>
@@ -1678,7 +1678,7 @@
       </x:c>
       <x:c r="G33" s="11"/>
       <x:c r="H33" s="11" t="str">
-        <x:v>${final_summary_report_type} = 'horeca'</x:v>
+        <x:v>string-length(normalize-space(${final_summary_report_type})) = 0 or ${final_summary_report_type} = 'horeca'</x:v>
       </x:c>
       <x:c r="I33" s="11"/>
       <x:c r="J33" s="11"/>
@@ -1774,7 +1774,7 @@
       </x:c>
       <x:c r="G37" s="11"/>
       <x:c r="H37" s="11" t="str">
-        <x:v>${final_summary_report_type} = 'horeca'</x:v>
+        <x:v>string-length(normalize-space(${final_summary_report_type})) = 0 or ${final_summary_report_type} = 'horeca'</x:v>
       </x:c>
       <x:c r="I37" s="11"/>
       <x:c r="J37" s="11"/>
@@ -1922,7 +1922,7 @@
       </x:c>
       <x:c r="G43" s="11"/>
       <x:c r="H43" s="11" t="str">
-        <x:v>${final_summary_report_type} = 'horeca'</x:v>
+        <x:v>string-length(normalize-space(${final_summary_report_type})) = 0 or ${final_summary_report_type} = 'horeca'</x:v>
       </x:c>
       <x:c r="I43" s="11"/>
       <x:c r="J43" s="11"/>
@@ -2070,7 +2070,7 @@
       </x:c>
       <x:c r="G49" s="11"/>
       <x:c r="H49" s="11" t="str">
-        <x:v>${final_summary_report_type} = 'horeca'</x:v>
+        <x:v>string-length(normalize-space(${final_summary_report_type})) = 0 or ${final_summary_report_type} = 'horeca'</x:v>
       </x:c>
       <x:c r="I49" s="11"/>
       <x:c r="J49" s="11"/>
@@ -2166,7 +2166,7 @@
       </x:c>
       <x:c r="G53" s="11"/>
       <x:c r="H53" s="11" t="str">
-        <x:v>${final_summary_report_type} = 'horeca'</x:v>
+        <x:v>string-length(normalize-space(${final_summary_report_type})) = 0 or ${final_summary_report_type} = 'horeca'</x:v>
       </x:c>
       <x:c r="I53" s="11"/>
       <x:c r="J53" s="11"/>
@@ -2262,7 +2262,7 @@
       </x:c>
       <x:c r="G57" s="11"/>
       <x:c r="H57" s="11" t="str">
-        <x:v>${final_summary_report_type} = 'horeca'</x:v>
+        <x:v>string-length(normalize-space(${final_summary_report_type})) = 0 or ${final_summary_report_type} = 'horeca'</x:v>
       </x:c>
       <x:c r="I57" s="11"/>
       <x:c r="J57" s="11"/>
@@ -2358,7 +2358,7 @@
       </x:c>
       <x:c r="G61" s="11"/>
       <x:c r="H61" s="11" t="str">
-        <x:v>${final_summary_report_type} = 'horeca'</x:v>
+        <x:v>string-length(normalize-space(${final_summary_report_type})) = 0 or ${final_summary_report_type} = 'horeca'</x:v>
       </x:c>
       <x:c r="I61" s="11"/>
       <x:c r="J61" s="11"/>
@@ -2506,7 +2506,7 @@
       </x:c>
       <x:c r="G67" s="11"/>
       <x:c r="H67" s="11" t="str">
-        <x:v>${final_summary_report_type} = 'horeca'</x:v>
+        <x:v>string-length(normalize-space(${final_summary_report_type})) = 0 or ${final_summary_report_type} = 'horeca'</x:v>
       </x:c>
       <x:c r="I67" s="11"/>
       <x:c r="J67" s="11"/>
@@ -2602,7 +2602,7 @@
       </x:c>
       <x:c r="G71" s="11"/>
       <x:c r="H71" s="11" t="str">
-        <x:v>${final_summary_report_type} = 'horeca'</x:v>
+        <x:v>string-length(normalize-space(${final_summary_report_type})) = 0 or ${final_summary_report_type} = 'horeca'</x:v>
       </x:c>
       <x:c r="I71" s="11"/>
       <x:c r="J71" s="11"/>
@@ -2698,7 +2698,7 @@
       </x:c>
       <x:c r="G75" s="11"/>
       <x:c r="H75" s="11" t="str">
-        <x:v>${final_summary_report_type} = 'horeca'</x:v>
+        <x:v>string-length(normalize-space(${final_summary_report_type})) = 0 or ${final_summary_report_type} = 'horeca'</x:v>
       </x:c>
       <x:c r="I75" s="11"/>
       <x:c r="J75" s="11"/>
@@ -4197,9 +4197,7 @@
         <x:v>field-list</x:v>
       </x:c>
       <x:c r="G133" s="11"/>
-      <x:c r="H133" s="11" t="str">
-        <x:v>${final_summary_report_type} = 'gt'</x:v>
-      </x:c>
+      <x:c r="H133" s="11"/>
       <x:c r="I133" s="11"/>
       <x:c r="J133" s="11"/>
       <x:c r="K133" s="11"/>
@@ -6491,7 +6489,7 @@
       </x:c>
       <x:c r="G222" s="11"/>
       <x:c r="H222" s="11" t="str">
-        <x:v>${final_summary_report_type} = 'horeca'</x:v>
+        <x:v>string-length(normalize-space(${final_summary_report_type})) = 0 or ${final_summary_report_type} = 'horeca'</x:v>
       </x:c>
       <x:c r="I222" s="11"/>
       <x:c r="J222" s="11"/>
@@ -7464,9 +7462,7 @@
         <x:v>field-list</x:v>
       </x:c>
       <x:c r="G260" s="11"/>
-      <x:c r="H260" s="11" t="str">
-        <x:v>${final_summary_report_type} = 'gt'</x:v>
-      </x:c>
+      <x:c r="H260" s="11"/>
       <x:c r="I260" s="11"/>
       <x:c r="J260" s="11"/>
       <x:c r="K260" s="11"/>
@@ -7645,9 +7641,7 @@
         <x:v>field-list</x:v>
       </x:c>
       <x:c r="G267" s="11"/>
-      <x:c r="H267" s="11" t="str">
-        <x:v>${final_summary_report_type} = 'gt'</x:v>
-      </x:c>
+      <x:c r="H267" s="11"/>
       <x:c r="I267" s="11"/>
       <x:c r="J267" s="11"/>
       <x:c r="K267" s="11"/>
@@ -7826,9 +7820,7 @@
         <x:v>field-list</x:v>
       </x:c>
       <x:c r="G274" s="11"/>
-      <x:c r="H274" s="11" t="str">
-        <x:v>${final_summary_report_type} = 'gt'</x:v>
-      </x:c>
+      <x:c r="H274" s="11"/>
       <x:c r="I274" s="11"/>
       <x:c r="J274" s="11"/>
       <x:c r="K274" s="11"/>
@@ -9065,7 +9057,7 @@
       </x:c>
       <x:c r="G322" s="11"/>
       <x:c r="H322" s="11" t="str">
-        <x:v>${final_summary_report_type} = 'gt'</x:v>
+        <x:v>string-length(normalize-space(${final_summary_report_type})) = 0 or ${final_summary_report_type} = 'gt'</x:v>
       </x:c>
       <x:c r="I322" s="11"/>
       <x:c r="J322" s="11"/>
@@ -9327,7 +9319,7 @@
       </x:c>
       <x:c r="G332" s="11"/>
       <x:c r="H332" s="11" t="str">
-        <x:v>${final_summary_report_type} = 'gt'</x:v>
+        <x:v>string-length(normalize-space(${final_summary_report_type})) = 0 or ${final_summary_report_type} = 'gt'</x:v>
       </x:c>
       <x:c r="I332" s="11"/>
       <x:c r="J332" s="11"/>
@@ -9508,7 +9500,7 @@
       </x:c>
       <x:c r="G339" s="11"/>
       <x:c r="H339" s="11" t="str">
-        <x:v>${final_summary_report_type} = 'gt'</x:v>
+        <x:v>string-length(normalize-space(${final_summary_report_type})) = 0 or ${final_summary_report_type} = 'gt'</x:v>
       </x:c>
       <x:c r="I339" s="11"/>
       <x:c r="J339" s="11"/>
@@ -9689,7 +9681,7 @@
       </x:c>
       <x:c r="G346" s="11"/>
       <x:c r="H346" s="11" t="str">
-        <x:v>${final_summary_report_type} = 'gt'</x:v>
+        <x:v>string-length(normalize-space(${final_summary_report_type})) = 0 or ${final_summary_report_type} = 'gt'</x:v>
       </x:c>
       <x:c r="I346" s="11"/>
       <x:c r="J346" s="11"/>
@@ -9870,7 +9862,7 @@
       </x:c>
       <x:c r="G353" s="11"/>
       <x:c r="H353" s="11" t="str">
-        <x:v>${final_summary_report_type} = 'gt'</x:v>
+        <x:v>string-length(normalize-space(${final_summary_report_type})) = 0 or ${final_summary_report_type} = 'gt'</x:v>
       </x:c>
       <x:c r="I353" s="11"/>
       <x:c r="J353" s="11"/>
@@ -10132,7 +10124,7 @@
       </x:c>
       <x:c r="G363" s="11"/>
       <x:c r="H363" s="11" t="str">
-        <x:v>${final_summary_report_type} = 'gt'</x:v>
+        <x:v>string-length(normalize-space(${final_summary_report_type})) = 0 or ${final_summary_report_type} = 'gt'</x:v>
       </x:c>
       <x:c r="I363" s="11"/>
       <x:c r="J363" s="11"/>
@@ -10313,7 +10305,7 @@
       </x:c>
       <x:c r="G370" s="11"/>
       <x:c r="H370" s="11" t="str">
-        <x:v>${final_summary_report_type} = 'gt'</x:v>
+        <x:v>string-length(normalize-space(${final_summary_report_type})) = 0 or ${final_summary_report_type} = 'gt'</x:v>
       </x:c>
       <x:c r="I370" s="11"/>
       <x:c r="J370" s="11"/>
@@ -10494,7 +10486,7 @@
       </x:c>
       <x:c r="G377" s="11"/>
       <x:c r="H377" s="11" t="str">
-        <x:v>${final_summary_report_type} = 'gt'</x:v>
+        <x:v>string-length(normalize-space(${final_summary_report_type})) = 0 or ${final_summary_report_type} = 'gt'</x:v>
       </x:c>
       <x:c r="I377" s="11"/>
       <x:c r="J377" s="11"/>
@@ -10756,7 +10748,7 @@
       </x:c>
       <x:c r="G387" s="11"/>
       <x:c r="H387" s="11" t="str">
-        <x:v>${final_summary_report_type} = 'gt'</x:v>
+        <x:v>string-length(normalize-space(${final_summary_report_type})) = 0 or ${final_summary_report_type} = 'gt'</x:v>
       </x:c>
       <x:c r="I387" s="11"/>
       <x:c r="J387" s="11"/>
@@ -10937,7 +10929,7 @@
       </x:c>
       <x:c r="G394" s="11"/>
       <x:c r="H394" s="11" t="str">
-        <x:v>${final_summary_report_type} = 'gt'</x:v>
+        <x:v>string-length(normalize-space(${final_summary_report_type})) = 0 or ${final_summary_report_type} = 'gt'</x:v>
       </x:c>
       <x:c r="I394" s="11"/>
       <x:c r="J394" s="11"/>
@@ -13790,7 +13782,7 @@
       </x:c>
       <x:c r="G505" s="11"/>
       <x:c r="H505" s="11" t="str">
-        <x:v>${final_summary_report_type} = 'gt'</x:v>
+        <x:v>string-length(normalize-space(${final_summary_report_type})) = 0 or ${final_summary_report_type} = 'gt'</x:v>
       </x:c>
       <x:c r="I505" s="11"/>
       <x:c r="J505" s="11"/>
@@ -14052,7 +14044,7 @@
       </x:c>
       <x:c r="G515" s="11"/>
       <x:c r="H515" s="11" t="str">
-        <x:v>${final_summary_report_type} = 'gt'</x:v>
+        <x:v>string-length(normalize-space(${final_summary_report_type})) = 0 or ${final_summary_report_type} = 'gt'</x:v>
       </x:c>
       <x:c r="I515" s="11"/>
       <x:c r="J515" s="11"/>
@@ -14233,7 +14225,7 @@
       </x:c>
       <x:c r="G522" s="11"/>
       <x:c r="H522" s="11" t="str">
-        <x:v>${final_summary_report_type} = 'gt'</x:v>
+        <x:v>string-length(normalize-space(${final_summary_report_type})) = 0 or ${final_summary_report_type} = 'gt'</x:v>
       </x:c>
       <x:c r="I522" s="11"/>
       <x:c r="J522" s="11"/>
@@ -14414,7 +14406,7 @@
       </x:c>
       <x:c r="G529" s="11"/>
       <x:c r="H529" s="11" t="str">
-        <x:v>${final_summary_report_type} = 'gt'</x:v>
+        <x:v>string-length(normalize-space(${final_summary_report_type})) = 0 or ${final_summary_report_type} = 'gt'</x:v>
       </x:c>
       <x:c r="I529" s="11"/>
       <x:c r="J529" s="11"/>
@@ -14595,7 +14587,7 @@
       </x:c>
       <x:c r="G536" s="11"/>
       <x:c r="H536" s="11" t="str">
-        <x:v>${final_summary_report_type} = 'gt'</x:v>
+        <x:v>string-length(normalize-space(${final_summary_report_type})) = 0 or ${final_summary_report_type} = 'gt'</x:v>
       </x:c>
       <x:c r="I536" s="11"/>
       <x:c r="J536" s="11"/>

</xml_diff>

<commit_message>
Route Kobo products after report type selection
</commit_message>
<xml_diff>
--- a/templates/KB_Market_Improvement_XLSForm_GT_HORECA.xlsx
+++ b/templates/KB_Market_Improvement_XLSForm_GT_HORECA.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="survey" sheetId="1" r:id="R4f44dbec69b94b5e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="choices" sheetId="2" r:id="Raf5f1cd1db71408e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="settings" sheetId="3" r:id="R0d2a0057f05a49b2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bot_Logic" sheetId="4" r:id="Rc547f61ed6d1488c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bot_Data_Map" sheetId="5" r:id="Ra90132a7a14c451a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="survey" sheetId="1" r:id="R656fd06bac004168"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="choices" sheetId="2" r:id="Re1688679d57a425a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="settings" sheetId="3" r:id="Rd6e944611b654d96"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bot_Logic" sheetId="4" r:id="R9595ba678a004b1d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bot_Data_Map" sheetId="5" r:id="R99663956829847bc"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1024,7 +1024,9 @@
       <x:c r="E6" s="11"/>
       <x:c r="F6" s="11"/>
       <x:c r="G6" s="11"/>
-      <x:c r="H6" s="11"/>
+      <x:c r="H6" s="11" t="str">
+        <x:v>(${final_summary_report_type} = 'gt' or ${final_summary_report_type} = 'horeca')</x:v>
+      </x:c>
       <x:c r="I6" s="11"/>
       <x:c r="J6" s="11"/>
       <x:c r="K6" s="11"/>
@@ -1045,7 +1047,9 @@
       <x:c r="E7" s="11"/>
       <x:c r="F7" s="11"/>
       <x:c r="G7" s="11"/>
-      <x:c r="H7" s="11"/>
+      <x:c r="H7" s="11" t="str">
+        <x:v>(${final_summary_report_type} = 'gt' or ${final_summary_report_type} = 'horeca')</x:v>
+      </x:c>
       <x:c r="I7" s="11" t="str">
         <x:v>. &gt;= 0</x:v>
       </x:c>
@@ -1070,7 +1074,9 @@
       <x:c r="E8" s="11"/>
       <x:c r="F8" s="11"/>
       <x:c r="G8" s="11"/>
-      <x:c r="H8" s="11"/>
+      <x:c r="H8" s="11" t="str">
+        <x:v>(${final_summary_report_type} = 'gt' or ${final_summary_report_type} = 'horeca')</x:v>
+      </x:c>
       <x:c r="I8" s="11" t="str">
         <x:v>. &gt;= 0</x:v>
       </x:c>
@@ -1097,7 +1103,9 @@
       </x:c>
       <x:c r="F9" s="11"/>
       <x:c r="G9" s="11"/>
-      <x:c r="H9" s="11"/>
+      <x:c r="H9" s="11" t="str">
+        <x:v>(${final_summary_report_type} = 'gt' or ${final_summary_report_type} = 'horeca')</x:v>
+      </x:c>
       <x:c r="I9" s="11"/>
       <x:c r="J9" s="11"/>
       <x:c r="K9" s="11"/>
@@ -1121,7 +1129,7 @@
       <x:c r="F10" s="11"/>
       <x:c r="G10" s="11"/>
       <x:c r="H10" s="11" t="str">
-        <x:v>not(normalize-space(${outlet_name}) = 'បូកសរុបរួម' or normalize-space(${outlet_name}) = 'បូកសរុបរូម' or normalize-space(${outlet_name}) = 'សរុបរួម' or normalize-space(${outlet_name}) = 'បួកសរុបរួម')</x:v>
+        <x:v>(${final_summary_report_type} = 'gt' or ${final_summary_report_type} = 'horeca') and (not(normalize-space(${outlet_name}) = 'បូកសរុបរួម' or normalize-space(${outlet_name}) = 'បូកសរុបរូម' or normalize-space(${outlet_name}) = 'សរុបរួម' or normalize-space(${outlet_name}) = 'បួកសរុបរួម'))</x:v>
       </x:c>
       <x:c r="I10" s="11"/>
       <x:c r="J10" s="11"/>
@@ -1144,7 +1152,7 @@
       <x:c r="F11" s="11"/>
       <x:c r="G11" s="11"/>
       <x:c r="H11" s="11" t="str">
-        <x:v>not(normalize-space(${outlet_name}) = 'បូកសរុបរួម' or normalize-space(${outlet_name}) = 'បូកសរុបរូម' or normalize-space(${outlet_name}) = 'សរុបរួម' or normalize-space(${outlet_name}) = 'បួកសរុបរួម')</x:v>
+        <x:v>(${final_summary_report_type} = 'gt' or ${final_summary_report_type} = 'horeca') and (not(normalize-space(${outlet_name}) = 'បូកសរុបរួម' or normalize-space(${outlet_name}) = 'បូកសរុបរូម' or normalize-space(${outlet_name}) = 'សរុបរួម' or normalize-space(${outlet_name}) = 'បួកសរុបរួម'))</x:v>
       </x:c>
       <x:c r="I11" s="11"/>
       <x:c r="J11" s="11"/>
@@ -1169,7 +1177,7 @@
       <x:c r="F12" s="11"/>
       <x:c r="G12" s="11"/>
       <x:c r="H12" s="11" t="str">
-        <x:v>not(normalize-space(${outlet_name}) = 'បូកសរុបរួម' or normalize-space(${outlet_name}) = 'បូកសរុបរូម' or normalize-space(${outlet_name}) = 'សរុបរួម' or normalize-space(${outlet_name}) = 'បួកសរុបរួម')</x:v>
+        <x:v>(${final_summary_report_type} = 'gt' or ${final_summary_report_type} = 'horeca') and (not(normalize-space(${outlet_name}) = 'បូកសរុបរួម' or normalize-space(${outlet_name}) = 'បូកសរុបរូម' or normalize-space(${outlet_name}) = 'សរុបរួម' or normalize-space(${outlet_name}) = 'បួកសរុបរួម'))</x:v>
       </x:c>
       <x:c r="I12" s="11"/>
       <x:c r="J12" s="11"/>
@@ -1196,7 +1204,7 @@
       <x:c r="F13" s="11"/>
       <x:c r="G13" s="11"/>
       <x:c r="H13" s="11" t="str">
-        <x:v>not(normalize-space(${outlet_name}) = 'បូកសរុបរួម' or normalize-space(${outlet_name}) = 'បូកសរុបរូម' or normalize-space(${outlet_name}) = 'សរុបរួម' or normalize-space(${outlet_name}) = 'បួកសរុបរួម')</x:v>
+        <x:v>(${final_summary_report_type} = 'gt' or ${final_summary_report_type} = 'horeca') and (not(normalize-space(${outlet_name}) = 'បូកសរុបរួម' or normalize-space(${outlet_name}) = 'បូកសរុបរូម' or normalize-space(${outlet_name}) = 'សរុបរួម' or normalize-space(${outlet_name}) = 'បួកសរុបរួម'))</x:v>
       </x:c>
       <x:c r="I13" s="11"/>
       <x:c r="J13" s="11"/>
@@ -1221,7 +1229,7 @@
       <x:c r="F14" s="11"/>
       <x:c r="G14" s="11"/>
       <x:c r="H14" s="11" t="str">
-        <x:v>not(normalize-space(${outlet_name}) = 'បូកសរុបរួម' or normalize-space(${outlet_name}) = 'បូកសរុបរូម' or normalize-space(${outlet_name}) = 'សរុបរួម' or normalize-space(${outlet_name}) = 'បួកសរុបរួម')</x:v>
+        <x:v>(${final_summary_report_type} = 'gt' or ${final_summary_report_type} = 'horeca') and (not(normalize-space(${outlet_name}) = 'បូកសរុបរួម' or normalize-space(${outlet_name}) = 'បូកសរុបរូម' or normalize-space(${outlet_name}) = 'សរុបរួម' or normalize-space(${outlet_name}) = 'បួកសរុបរួម'))</x:v>
       </x:c>
       <x:c r="I14" s="11"/>
       <x:c r="J14" s="11"/>
@@ -1250,7 +1258,7 @@
         <x:v>contains(report_scope, ${final_summary_report_type})</x:v>
       </x:c>
       <x:c r="H15" s="11" t="str">
-        <x:v>not(normalize-space(${outlet_name}) = 'បូកសរុបរួម' or normalize-space(${outlet_name}) = 'បូកសរុបរូម' or normalize-space(${outlet_name}) = 'សរុបរួម' or normalize-space(${outlet_name}) = 'បួកសរុបរួម')</x:v>
+        <x:v>(${final_summary_report_type} = 'gt' or ${final_summary_report_type} = 'horeca') and (not(normalize-space(${outlet_name}) = 'បូកសរុបរួម' or normalize-space(${outlet_name}) = 'បូកសរុបរូម' or normalize-space(${outlet_name}) = 'សរុបរួម' or normalize-space(${outlet_name}) = 'បួកសរុបរួម'))</x:v>
       </x:c>
       <x:c r="I15" s="11"/>
       <x:c r="J15" s="11"/>
@@ -1277,7 +1285,7 @@
       </x:c>
       <x:c r="G16" s="11"/>
       <x:c r="H16" s="11" t="str">
-        <x:v>not(normalize-space(${outlet_name}) = 'បូកសរុបរួម' or normalize-space(${outlet_name}) = 'បូកសរុបរូម' or normalize-space(${outlet_name}) = 'សរុបរួម' or normalize-space(${outlet_name}) = 'បួកសរុបរួម')</x:v>
+        <x:v>(${final_summary_report_type} = 'gt' or ${final_summary_report_type} = 'horeca') and (not(normalize-space(${outlet_name}) = 'បូកសរុបរួម' or normalize-space(${outlet_name}) = 'បូកសរុបរូម' or normalize-space(${outlet_name}) = 'សរុបរួម' or normalize-space(${outlet_name}) = 'បួកសរុបរួម'))</x:v>
       </x:c>
       <x:c r="I16" s="11"/>
       <x:c r="J16" s="11"/>
@@ -1301,7 +1309,9 @@
       </x:c>
       <x:c r="F17" s="11"/>
       <x:c r="G17" s="11"/>
-      <x:c r="H17" s="11"/>
+      <x:c r="H17" s="11" t="str">
+        <x:v>(${final_summary_report_type} = 'gt' or ${final_summary_report_type} = 'horeca')</x:v>
+      </x:c>
       <x:c r="I17" s="11"/>
       <x:c r="J17" s="11"/>
       <x:c r="K17" s="11"/>
@@ -1340,7 +1350,7 @@
       <x:c r="F19" s="11"/>
       <x:c r="G19" s="11"/>
       <x:c r="H19" s="11" t="str">
-        <x:v>not(normalize-space(${outlet_name}) = 'បូកសរុបរួម' or normalize-space(${outlet_name}) = 'បូកសរុបរូម' or normalize-space(${outlet_name}) = 'សរុបរួម' or normalize-space(${outlet_name}) = 'បួកសរុបរួម')</x:v>
+        <x:v>(${final_summary_report_type} = 'gt' or ${final_summary_report_type} = 'horeca') and (not(normalize-space(${outlet_name}) = 'បូកសរុបរួម' or normalize-space(${outlet_name}) = 'បូកសរុបរូម' or normalize-space(${outlet_name}) = 'សរុបរួម' or normalize-space(${outlet_name}) = 'បួកសរុបរួម'))</x:v>
       </x:c>
       <x:c r="I19" s="11"/>
       <x:c r="J19" s="11"/>
@@ -1434,7 +1444,7 @@
       </x:c>
       <x:c r="G23" s="11"/>
       <x:c r="H23" s="11" t="str">
-        <x:v>string-length(normalize-space(${final_summary_report_type})) = 0 or ${final_summary_report_type} = 'horeca'</x:v>
+        <x:v>${final_summary_report_type} = 'horeca'</x:v>
       </x:c>
       <x:c r="I23" s="11"/>
       <x:c r="J23" s="11"/>
@@ -1582,7 +1592,7 @@
       </x:c>
       <x:c r="G29" s="11"/>
       <x:c r="H29" s="11" t="str">
-        <x:v>string-length(normalize-space(${final_summary_report_type})) = 0 or ${final_summary_report_type} = 'horeca'</x:v>
+        <x:v>${final_summary_report_type} = 'horeca'</x:v>
       </x:c>
       <x:c r="I29" s="11"/>
       <x:c r="J29" s="11"/>
@@ -1678,7 +1688,7 @@
       </x:c>
       <x:c r="G33" s="11"/>
       <x:c r="H33" s="11" t="str">
-        <x:v>string-length(normalize-space(${final_summary_report_type})) = 0 or ${final_summary_report_type} = 'horeca'</x:v>
+        <x:v>${final_summary_report_type} = 'horeca'</x:v>
       </x:c>
       <x:c r="I33" s="11"/>
       <x:c r="J33" s="11"/>
@@ -1774,7 +1784,7 @@
       </x:c>
       <x:c r="G37" s="11"/>
       <x:c r="H37" s="11" t="str">
-        <x:v>string-length(normalize-space(${final_summary_report_type})) = 0 or ${final_summary_report_type} = 'horeca'</x:v>
+        <x:v>${final_summary_report_type} = 'horeca'</x:v>
       </x:c>
       <x:c r="I37" s="11"/>
       <x:c r="J37" s="11"/>
@@ -1922,7 +1932,7 @@
       </x:c>
       <x:c r="G43" s="11"/>
       <x:c r="H43" s="11" t="str">
-        <x:v>string-length(normalize-space(${final_summary_report_type})) = 0 or ${final_summary_report_type} = 'horeca'</x:v>
+        <x:v>${final_summary_report_type} = 'horeca'</x:v>
       </x:c>
       <x:c r="I43" s="11"/>
       <x:c r="J43" s="11"/>
@@ -2070,7 +2080,7 @@
       </x:c>
       <x:c r="G49" s="11"/>
       <x:c r="H49" s="11" t="str">
-        <x:v>string-length(normalize-space(${final_summary_report_type})) = 0 or ${final_summary_report_type} = 'horeca'</x:v>
+        <x:v>${final_summary_report_type} = 'horeca'</x:v>
       </x:c>
       <x:c r="I49" s="11"/>
       <x:c r="J49" s="11"/>
@@ -2166,7 +2176,7 @@
       </x:c>
       <x:c r="G53" s="11"/>
       <x:c r="H53" s="11" t="str">
-        <x:v>string-length(normalize-space(${final_summary_report_type})) = 0 or ${final_summary_report_type} = 'horeca'</x:v>
+        <x:v>${final_summary_report_type} = 'horeca'</x:v>
       </x:c>
       <x:c r="I53" s="11"/>
       <x:c r="J53" s="11"/>
@@ -2262,7 +2272,7 @@
       </x:c>
       <x:c r="G57" s="11"/>
       <x:c r="H57" s="11" t="str">
-        <x:v>string-length(normalize-space(${final_summary_report_type})) = 0 or ${final_summary_report_type} = 'horeca'</x:v>
+        <x:v>${final_summary_report_type} = 'horeca'</x:v>
       </x:c>
       <x:c r="I57" s="11"/>
       <x:c r="J57" s="11"/>
@@ -2358,7 +2368,7 @@
       </x:c>
       <x:c r="G61" s="11"/>
       <x:c r="H61" s="11" t="str">
-        <x:v>string-length(normalize-space(${final_summary_report_type})) = 0 or ${final_summary_report_type} = 'horeca'</x:v>
+        <x:v>${final_summary_report_type} = 'horeca'</x:v>
       </x:c>
       <x:c r="I61" s="11"/>
       <x:c r="J61" s="11"/>
@@ -2506,7 +2516,7 @@
       </x:c>
       <x:c r="G67" s="11"/>
       <x:c r="H67" s="11" t="str">
-        <x:v>string-length(normalize-space(${final_summary_report_type})) = 0 or ${final_summary_report_type} = 'horeca'</x:v>
+        <x:v>${final_summary_report_type} = 'horeca'</x:v>
       </x:c>
       <x:c r="I67" s="11"/>
       <x:c r="J67" s="11"/>
@@ -2602,7 +2612,7 @@
       </x:c>
       <x:c r="G71" s="11"/>
       <x:c r="H71" s="11" t="str">
-        <x:v>string-length(normalize-space(${final_summary_report_type})) = 0 or ${final_summary_report_type} = 'horeca'</x:v>
+        <x:v>${final_summary_report_type} = 'horeca'</x:v>
       </x:c>
       <x:c r="I71" s="11"/>
       <x:c r="J71" s="11"/>
@@ -2698,7 +2708,7 @@
       </x:c>
       <x:c r="G75" s="11"/>
       <x:c r="H75" s="11" t="str">
-        <x:v>string-length(normalize-space(${final_summary_report_type})) = 0 or ${final_summary_report_type} = 'horeca'</x:v>
+        <x:v>${final_summary_report_type} = 'horeca'</x:v>
       </x:c>
       <x:c r="I75" s="11"/>
       <x:c r="J75" s="11"/>
@@ -2793,7 +2803,9 @@
         <x:v>field-list</x:v>
       </x:c>
       <x:c r="G79" s="11"/>
-      <x:c r="H79" s="11"/>
+      <x:c r="H79" s="11" t="str">
+        <x:v>(${final_summary_report_type} = 'gt' or ${final_summary_report_type} = 'horeca')</x:v>
+      </x:c>
       <x:c r="I79" s="11"/>
       <x:c r="J79" s="11"/>
       <x:c r="K79" s="11"/>
@@ -3082,7 +3094,9 @@
         <x:v>field-list</x:v>
       </x:c>
       <x:c r="G90" s="11"/>
-      <x:c r="H90" s="11"/>
+      <x:c r="H90" s="11" t="str">
+        <x:v>(${final_summary_report_type} = 'gt' or ${final_summary_report_type} = 'horeca')</x:v>
+      </x:c>
       <x:c r="I90" s="11"/>
       <x:c r="J90" s="11"/>
       <x:c r="K90" s="11"/>
@@ -3261,7 +3275,9 @@
         <x:v>field-list</x:v>
       </x:c>
       <x:c r="G97" s="11"/>
-      <x:c r="H97" s="11"/>
+      <x:c r="H97" s="11" t="str">
+        <x:v>(${final_summary_report_type} = 'gt' or ${final_summary_report_type} = 'horeca')</x:v>
+      </x:c>
       <x:c r="I97" s="11"/>
       <x:c r="J97" s="11"/>
       <x:c r="K97" s="11"/>
@@ -3440,7 +3456,9 @@
         <x:v>field-list</x:v>
       </x:c>
       <x:c r="G104" s="11"/>
-      <x:c r="H104" s="11"/>
+      <x:c r="H104" s="11" t="str">
+        <x:v>(${final_summary_report_type} = 'gt' or ${final_summary_report_type} = 'horeca')</x:v>
+      </x:c>
       <x:c r="I104" s="11"/>
       <x:c r="J104" s="11"/>
       <x:c r="K104" s="11"/>
@@ -3619,7 +3637,9 @@
         <x:v>field-list</x:v>
       </x:c>
       <x:c r="G111" s="11"/>
-      <x:c r="H111" s="11"/>
+      <x:c r="H111" s="11" t="str">
+        <x:v>(${final_summary_report_type} = 'gt' or ${final_summary_report_type} = 'horeca')</x:v>
+      </x:c>
       <x:c r="I111" s="11"/>
       <x:c r="J111" s="11"/>
       <x:c r="K111" s="11"/>
@@ -3908,7 +3928,9 @@
         <x:v>field-list</x:v>
       </x:c>
       <x:c r="G122" s="11"/>
-      <x:c r="H122" s="11"/>
+      <x:c r="H122" s="11" t="str">
+        <x:v>(${final_summary_report_type} = 'gt' or ${final_summary_report_type} = 'horeca')</x:v>
+      </x:c>
       <x:c r="I122" s="11"/>
       <x:c r="J122" s="11"/>
       <x:c r="K122" s="11"/>
@@ -4197,7 +4219,9 @@
         <x:v>field-list</x:v>
       </x:c>
       <x:c r="G133" s="11"/>
-      <x:c r="H133" s="11"/>
+      <x:c r="H133" s="11" t="str">
+        <x:v>(${final_summary_report_type} = 'gt' or ${final_summary_report_type} = 'horeca')</x:v>
+      </x:c>
       <x:c r="I133" s="11"/>
       <x:c r="J133" s="11"/>
       <x:c r="K133" s="11"/>
@@ -4486,7 +4510,9 @@
         <x:v>field-list</x:v>
       </x:c>
       <x:c r="G144" s="11"/>
-      <x:c r="H144" s="11"/>
+      <x:c r="H144" s="11" t="str">
+        <x:v>(${final_summary_report_type} = 'gt' or ${final_summary_report_type} = 'horeca')</x:v>
+      </x:c>
       <x:c r="I144" s="11"/>
       <x:c r="J144" s="11"/>
       <x:c r="K144" s="11"/>
@@ -4665,7 +4691,9 @@
         <x:v>field-list</x:v>
       </x:c>
       <x:c r="G151" s="11"/>
-      <x:c r="H151" s="11"/>
+      <x:c r="H151" s="11" t="str">
+        <x:v>(${final_summary_report_type} = 'gt' or ${final_summary_report_type} = 'horeca')</x:v>
+      </x:c>
       <x:c r="I151" s="11"/>
       <x:c r="J151" s="11"/>
       <x:c r="K151" s="11"/>
@@ -4844,7 +4872,9 @@
         <x:v>field-list</x:v>
       </x:c>
       <x:c r="G158" s="11"/>
-      <x:c r="H158" s="11"/>
+      <x:c r="H158" s="11" t="str">
+        <x:v>(${final_summary_report_type} = 'gt' or ${final_summary_report_type} = 'horeca')</x:v>
+      </x:c>
       <x:c r="I158" s="11"/>
       <x:c r="J158" s="11"/>
       <x:c r="K158" s="11"/>
@@ -5023,7 +5053,9 @@
         <x:v>field-list</x:v>
       </x:c>
       <x:c r="G165" s="11"/>
-      <x:c r="H165" s="11"/>
+      <x:c r="H165" s="11" t="str">
+        <x:v>(${final_summary_report_type} = 'gt' or ${final_summary_report_type} = 'horeca')</x:v>
+      </x:c>
       <x:c r="I165" s="11"/>
       <x:c r="J165" s="11"/>
       <x:c r="K165" s="11"/>
@@ -5202,7 +5234,9 @@
         <x:v>field-list</x:v>
       </x:c>
       <x:c r="G172" s="11"/>
-      <x:c r="H172" s="11"/>
+      <x:c r="H172" s="11" t="str">
+        <x:v>(${final_summary_report_type} = 'gt' or ${final_summary_report_type} = 'horeca')</x:v>
+      </x:c>
       <x:c r="I172" s="11"/>
       <x:c r="J172" s="11"/>
       <x:c r="K172" s="11"/>
@@ -5381,7 +5415,9 @@
         <x:v>field-list</x:v>
       </x:c>
       <x:c r="G179" s="11"/>
-      <x:c r="H179" s="11"/>
+      <x:c r="H179" s="11" t="str">
+        <x:v>(${final_summary_report_type} = 'gt' or ${final_summary_report_type} = 'horeca')</x:v>
+      </x:c>
       <x:c r="I179" s="11"/>
       <x:c r="J179" s="11"/>
       <x:c r="K179" s="11"/>
@@ -5560,7 +5596,9 @@
         <x:v>field-list</x:v>
       </x:c>
       <x:c r="G186" s="11"/>
-      <x:c r="H186" s="11"/>
+      <x:c r="H186" s="11" t="str">
+        <x:v>(${final_summary_report_type} = 'gt' or ${final_summary_report_type} = 'horeca')</x:v>
+      </x:c>
       <x:c r="I186" s="11"/>
       <x:c r="J186" s="11"/>
       <x:c r="K186" s="11"/>
@@ -5849,7 +5887,9 @@
         <x:v>field-list</x:v>
       </x:c>
       <x:c r="G197" s="11"/>
-      <x:c r="H197" s="11"/>
+      <x:c r="H197" s="11" t="str">
+        <x:v>(${final_summary_report_type} = 'gt' or ${final_summary_report_type} = 'horeca')</x:v>
+      </x:c>
       <x:c r="I197" s="11"/>
       <x:c r="J197" s="11"/>
       <x:c r="K197" s="11"/>
@@ -6049,7 +6089,9 @@
         <x:v>field-list</x:v>
       </x:c>
       <x:c r="G205" s="11"/>
-      <x:c r="H205" s="11"/>
+      <x:c r="H205" s="11" t="str">
+        <x:v>(${final_summary_report_type} = 'gt' or ${final_summary_report_type} = 'horeca')</x:v>
+      </x:c>
       <x:c r="I205" s="11"/>
       <x:c r="J205" s="11"/>
       <x:c r="K205" s="11"/>
@@ -6309,7 +6351,9 @@
         <x:v>field-list</x:v>
       </x:c>
       <x:c r="G215" s="11"/>
-      <x:c r="H215" s="11"/>
+      <x:c r="H215" s="11" t="str">
+        <x:v>(${final_summary_report_type} = 'gt' or ${final_summary_report_type} = 'horeca')</x:v>
+      </x:c>
       <x:c r="I215" s="11"/>
       <x:c r="J215" s="11"/>
       <x:c r="K215" s="11"/>
@@ -6489,7 +6533,7 @@
       </x:c>
       <x:c r="G222" s="11"/>
       <x:c r="H222" s="11" t="str">
-        <x:v>string-length(normalize-space(${final_summary_report_type})) = 0 or ${final_summary_report_type} = 'horeca'</x:v>
+        <x:v>${final_summary_report_type} = 'horeca'</x:v>
       </x:c>
       <x:c r="I222" s="11"/>
       <x:c r="J222" s="11"/>
@@ -6584,7 +6628,9 @@
         <x:v>field-list</x:v>
       </x:c>
       <x:c r="G226" s="11"/>
-      <x:c r="H226" s="11"/>
+      <x:c r="H226" s="11" t="str">
+        <x:v>(${final_summary_report_type} = 'gt' or ${final_summary_report_type} = 'horeca')</x:v>
+      </x:c>
       <x:c r="I226" s="11"/>
       <x:c r="J226" s="11"/>
       <x:c r="K226" s="11"/>
@@ -6844,7 +6890,9 @@
         <x:v>field-list</x:v>
       </x:c>
       <x:c r="G236" s="11"/>
-      <x:c r="H236" s="11"/>
+      <x:c r="H236" s="11" t="str">
+        <x:v>(${final_summary_report_type} = 'gt' or ${final_summary_report_type} = 'horeca')</x:v>
+      </x:c>
       <x:c r="I236" s="11"/>
       <x:c r="J236" s="11"/>
       <x:c r="K236" s="11"/>
@@ -7023,7 +7071,9 @@
         <x:v>field-list</x:v>
       </x:c>
       <x:c r="G243" s="11"/>
-      <x:c r="H243" s="11"/>
+      <x:c r="H243" s="11" t="str">
+        <x:v>(${final_summary_report_type} = 'gt' or ${final_summary_report_type} = 'horeca')</x:v>
+      </x:c>
       <x:c r="I243" s="11"/>
       <x:c r="J243" s="11"/>
       <x:c r="K243" s="11"/>
@@ -7202,7 +7252,9 @@
         <x:v>field-list</x:v>
       </x:c>
       <x:c r="G250" s="11"/>
-      <x:c r="H250" s="11"/>
+      <x:c r="H250" s="11" t="str">
+        <x:v>(${final_summary_report_type} = 'gt' or ${final_summary_report_type} = 'horeca')</x:v>
+      </x:c>
       <x:c r="I250" s="11"/>
       <x:c r="J250" s="11"/>
       <x:c r="K250" s="11"/>
@@ -7462,7 +7514,9 @@
         <x:v>field-list</x:v>
       </x:c>
       <x:c r="G260" s="11"/>
-      <x:c r="H260" s="11"/>
+      <x:c r="H260" s="11" t="str">
+        <x:v>(${final_summary_report_type} = 'gt' or ${final_summary_report_type} = 'horeca')</x:v>
+      </x:c>
       <x:c r="I260" s="11"/>
       <x:c r="J260" s="11"/>
       <x:c r="K260" s="11"/>
@@ -7641,7 +7695,9 @@
         <x:v>field-list</x:v>
       </x:c>
       <x:c r="G267" s="11"/>
-      <x:c r="H267" s="11"/>
+      <x:c r="H267" s="11" t="str">
+        <x:v>(${final_summary_report_type} = 'gt' or ${final_summary_report_type} = 'horeca')</x:v>
+      </x:c>
       <x:c r="I267" s="11"/>
       <x:c r="J267" s="11"/>
       <x:c r="K267" s="11"/>
@@ -7820,7 +7876,9 @@
         <x:v>field-list</x:v>
       </x:c>
       <x:c r="G274" s="11"/>
-      <x:c r="H274" s="11"/>
+      <x:c r="H274" s="11" t="str">
+        <x:v>(${final_summary_report_type} = 'gt' or ${final_summary_report_type} = 'horeca')</x:v>
+      </x:c>
       <x:c r="I274" s="11"/>
       <x:c r="J274" s="11"/>
       <x:c r="K274" s="11"/>
@@ -7999,7 +8057,9 @@
         <x:v>field-list</x:v>
       </x:c>
       <x:c r="G281" s="11"/>
-      <x:c r="H281" s="11"/>
+      <x:c r="H281" s="11" t="str">
+        <x:v>(${final_summary_report_type} = 'gt' or ${final_summary_report_type} = 'horeca')</x:v>
+      </x:c>
       <x:c r="I281" s="11"/>
       <x:c r="J281" s="11"/>
       <x:c r="K281" s="11"/>
@@ -8259,7 +8319,9 @@
         <x:v>field-list</x:v>
       </x:c>
       <x:c r="G291" s="11"/>
-      <x:c r="H291" s="11"/>
+      <x:c r="H291" s="11" t="str">
+        <x:v>(${final_summary_report_type} = 'gt' or ${final_summary_report_type} = 'horeca')</x:v>
+      </x:c>
       <x:c r="I291" s="11"/>
       <x:c r="J291" s="11"/>
       <x:c r="K291" s="11"/>
@@ -8438,7 +8500,9 @@
         <x:v>field-list</x:v>
       </x:c>
       <x:c r="G298" s="11"/>
-      <x:c r="H298" s="11"/>
+      <x:c r="H298" s="11" t="str">
+        <x:v>(${final_summary_report_type} = 'gt' or ${final_summary_report_type} = 'horeca')</x:v>
+      </x:c>
       <x:c r="I298" s="11"/>
       <x:c r="J298" s="11"/>
       <x:c r="K298" s="11"/>
@@ -8617,7 +8681,9 @@
         <x:v>field-list</x:v>
       </x:c>
       <x:c r="G305" s="11"/>
-      <x:c r="H305" s="11"/>
+      <x:c r="H305" s="11" t="str">
+        <x:v>(${final_summary_report_type} = 'gt' or ${final_summary_report_type} = 'horeca')</x:v>
+      </x:c>
       <x:c r="I305" s="11"/>
       <x:c r="J305" s="11"/>
       <x:c r="K305" s="11"/>
@@ -8877,7 +8943,9 @@
         <x:v>field-list</x:v>
       </x:c>
       <x:c r="G315" s="11"/>
-      <x:c r="H315" s="11"/>
+      <x:c r="H315" s="11" t="str">
+        <x:v>(${final_summary_report_type} = 'gt' or ${final_summary_report_type} = 'horeca')</x:v>
+      </x:c>
       <x:c r="I315" s="11"/>
       <x:c r="J315" s="11"/>
       <x:c r="K315" s="11"/>
@@ -9057,7 +9125,7 @@
       </x:c>
       <x:c r="G322" s="11"/>
       <x:c r="H322" s="11" t="str">
-        <x:v>string-length(normalize-space(${final_summary_report_type})) = 0 or ${final_summary_report_type} = 'gt'</x:v>
+        <x:v>${final_summary_report_type} = 'gt'</x:v>
       </x:c>
       <x:c r="I322" s="11"/>
       <x:c r="J322" s="11"/>
@@ -9319,7 +9387,7 @@
       </x:c>
       <x:c r="G332" s="11"/>
       <x:c r="H332" s="11" t="str">
-        <x:v>string-length(normalize-space(${final_summary_report_type})) = 0 or ${final_summary_report_type} = 'gt'</x:v>
+        <x:v>${final_summary_report_type} = 'gt'</x:v>
       </x:c>
       <x:c r="I332" s="11"/>
       <x:c r="J332" s="11"/>
@@ -9500,7 +9568,7 @@
       </x:c>
       <x:c r="G339" s="11"/>
       <x:c r="H339" s="11" t="str">
-        <x:v>string-length(normalize-space(${final_summary_report_type})) = 0 or ${final_summary_report_type} = 'gt'</x:v>
+        <x:v>${final_summary_report_type} = 'gt'</x:v>
       </x:c>
       <x:c r="I339" s="11"/>
       <x:c r="J339" s="11"/>
@@ -9681,7 +9749,7 @@
       </x:c>
       <x:c r="G346" s="11"/>
       <x:c r="H346" s="11" t="str">
-        <x:v>string-length(normalize-space(${final_summary_report_type})) = 0 or ${final_summary_report_type} = 'gt'</x:v>
+        <x:v>${final_summary_report_type} = 'gt'</x:v>
       </x:c>
       <x:c r="I346" s="11"/>
       <x:c r="J346" s="11"/>
@@ -9862,7 +9930,7 @@
       </x:c>
       <x:c r="G353" s="11"/>
       <x:c r="H353" s="11" t="str">
-        <x:v>string-length(normalize-space(${final_summary_report_type})) = 0 or ${final_summary_report_type} = 'gt'</x:v>
+        <x:v>${final_summary_report_type} = 'gt'</x:v>
       </x:c>
       <x:c r="I353" s="11"/>
       <x:c r="J353" s="11"/>
@@ -10124,7 +10192,7 @@
       </x:c>
       <x:c r="G363" s="11"/>
       <x:c r="H363" s="11" t="str">
-        <x:v>string-length(normalize-space(${final_summary_report_type})) = 0 or ${final_summary_report_type} = 'gt'</x:v>
+        <x:v>${final_summary_report_type} = 'gt'</x:v>
       </x:c>
       <x:c r="I363" s="11"/>
       <x:c r="J363" s="11"/>
@@ -10305,7 +10373,7 @@
       </x:c>
       <x:c r="G370" s="11"/>
       <x:c r="H370" s="11" t="str">
-        <x:v>string-length(normalize-space(${final_summary_report_type})) = 0 or ${final_summary_report_type} = 'gt'</x:v>
+        <x:v>${final_summary_report_type} = 'gt'</x:v>
       </x:c>
       <x:c r="I370" s="11"/>
       <x:c r="J370" s="11"/>
@@ -10486,7 +10554,7 @@
       </x:c>
       <x:c r="G377" s="11"/>
       <x:c r="H377" s="11" t="str">
-        <x:v>string-length(normalize-space(${final_summary_report_type})) = 0 or ${final_summary_report_type} = 'gt'</x:v>
+        <x:v>${final_summary_report_type} = 'gt'</x:v>
       </x:c>
       <x:c r="I377" s="11"/>
       <x:c r="J377" s="11"/>
@@ -10748,7 +10816,7 @@
       </x:c>
       <x:c r="G387" s="11"/>
       <x:c r="H387" s="11" t="str">
-        <x:v>string-length(normalize-space(${final_summary_report_type})) = 0 or ${final_summary_report_type} = 'gt'</x:v>
+        <x:v>${final_summary_report_type} = 'gt'</x:v>
       </x:c>
       <x:c r="I387" s="11"/>
       <x:c r="J387" s="11"/>
@@ -10929,7 +10997,7 @@
       </x:c>
       <x:c r="G394" s="11"/>
       <x:c r="H394" s="11" t="str">
-        <x:v>string-length(normalize-space(${final_summary_report_type})) = 0 or ${final_summary_report_type} = 'gt'</x:v>
+        <x:v>${final_summary_report_type} = 'gt'</x:v>
       </x:c>
       <x:c r="I394" s="11"/>
       <x:c r="J394" s="11"/>
@@ -11109,7 +11177,9 @@
         <x:v>field-list</x:v>
       </x:c>
       <x:c r="G401" s="11"/>
-      <x:c r="H401" s="11"/>
+      <x:c r="H401" s="11" t="str">
+        <x:v>(${final_summary_report_type} = 'gt' or ${final_summary_report_type} = 'horeca')</x:v>
+      </x:c>
       <x:c r="I401" s="11"/>
       <x:c r="J401" s="11"/>
       <x:c r="K401" s="11"/>
@@ -11369,7 +11439,9 @@
         <x:v>field-list</x:v>
       </x:c>
       <x:c r="G411" s="11"/>
-      <x:c r="H411" s="11"/>
+      <x:c r="H411" s="11" t="str">
+        <x:v>(${final_summary_report_type} = 'gt' or ${final_summary_report_type} = 'horeca')</x:v>
+      </x:c>
       <x:c r="I411" s="11"/>
       <x:c r="J411" s="11"/>
       <x:c r="K411" s="11"/>
@@ -11548,7 +11620,9 @@
         <x:v>field-list</x:v>
       </x:c>
       <x:c r="G418" s="11"/>
-      <x:c r="H418" s="11"/>
+      <x:c r="H418" s="11" t="str">
+        <x:v>(${final_summary_report_type} = 'gt' or ${final_summary_report_type} = 'horeca')</x:v>
+      </x:c>
       <x:c r="I418" s="11"/>
       <x:c r="J418" s="11"/>
       <x:c r="K418" s="11"/>
@@ -11727,7 +11801,9 @@
         <x:v>field-list</x:v>
       </x:c>
       <x:c r="G425" s="11"/>
-      <x:c r="H425" s="11"/>
+      <x:c r="H425" s="11" t="str">
+        <x:v>(${final_summary_report_type} = 'gt' or ${final_summary_report_type} = 'horeca')</x:v>
+      </x:c>
       <x:c r="I425" s="11"/>
       <x:c r="J425" s="11"/>
       <x:c r="K425" s="11"/>
@@ -11906,7 +11982,9 @@
         <x:v>field-list</x:v>
       </x:c>
       <x:c r="G432" s="11"/>
-      <x:c r="H432" s="11"/>
+      <x:c r="H432" s="11" t="str">
+        <x:v>(${final_summary_report_type} = 'gt' or ${final_summary_report_type} = 'horeca')</x:v>
+      </x:c>
       <x:c r="I432" s="11"/>
       <x:c r="J432" s="11"/>
       <x:c r="K432" s="11"/>
@@ -12166,7 +12244,9 @@
         <x:v>field-list</x:v>
       </x:c>
       <x:c r="G442" s="11"/>
-      <x:c r="H442" s="11"/>
+      <x:c r="H442" s="11" t="str">
+        <x:v>(${final_summary_report_type} = 'gt' or ${final_summary_report_type} = 'horeca')</x:v>
+      </x:c>
       <x:c r="I442" s="11"/>
       <x:c r="J442" s="11"/>
       <x:c r="K442" s="11"/>
@@ -12426,7 +12506,9 @@
         <x:v>field-list</x:v>
       </x:c>
       <x:c r="G452" s="11"/>
-      <x:c r="H452" s="11"/>
+      <x:c r="H452" s="11" t="str">
+        <x:v>(${final_summary_report_type} = 'gt' or ${final_summary_report_type} = 'horeca')</x:v>
+      </x:c>
       <x:c r="I452" s="11"/>
       <x:c r="J452" s="11"/>
       <x:c r="K452" s="11"/>
@@ -12605,7 +12687,9 @@
         <x:v>field-list</x:v>
       </x:c>
       <x:c r="G459" s="11"/>
-      <x:c r="H459" s="11"/>
+      <x:c r="H459" s="11" t="str">
+        <x:v>(${final_summary_report_type} = 'gt' or ${final_summary_report_type} = 'horeca')</x:v>
+      </x:c>
       <x:c r="I459" s="11"/>
       <x:c r="J459" s="11"/>
       <x:c r="K459" s="11"/>
@@ -12805,7 +12889,9 @@
         <x:v>field-list</x:v>
       </x:c>
       <x:c r="G467" s="11"/>
-      <x:c r="H467" s="11"/>
+      <x:c r="H467" s="11" t="str">
+        <x:v>(${final_summary_report_type} = 'gt' or ${final_summary_report_type} = 'horeca')</x:v>
+      </x:c>
       <x:c r="I467" s="11"/>
       <x:c r="J467" s="11"/>
       <x:c r="K467" s="11"/>
@@ -13065,7 +13151,9 @@
         <x:v>field-list</x:v>
       </x:c>
       <x:c r="G477" s="11"/>
-      <x:c r="H477" s="11"/>
+      <x:c r="H477" s="11" t="str">
+        <x:v>(${final_summary_report_type} = 'gt' or ${final_summary_report_type} = 'horeca')</x:v>
+      </x:c>
       <x:c r="I477" s="11"/>
       <x:c r="J477" s="11"/>
       <x:c r="K477" s="11"/>
@@ -13244,7 +13332,9 @@
         <x:v>field-list</x:v>
       </x:c>
       <x:c r="G484" s="11"/>
-      <x:c r="H484" s="11"/>
+      <x:c r="H484" s="11" t="str">
+        <x:v>(${final_summary_report_type} = 'gt' or ${final_summary_report_type} = 'horeca')</x:v>
+      </x:c>
       <x:c r="I484" s="11"/>
       <x:c r="J484" s="11"/>
       <x:c r="K484" s="11"/>
@@ -13423,7 +13513,9 @@
         <x:v>field-list</x:v>
       </x:c>
       <x:c r="G491" s="11"/>
-      <x:c r="H491" s="11"/>
+      <x:c r="H491" s="11" t="str">
+        <x:v>(${final_summary_report_type} = 'gt' or ${final_summary_report_type} = 'horeca')</x:v>
+      </x:c>
       <x:c r="I491" s="11"/>
       <x:c r="J491" s="11"/>
       <x:c r="K491" s="11"/>
@@ -13602,7 +13694,9 @@
         <x:v>field-list</x:v>
       </x:c>
       <x:c r="G498" s="11"/>
-      <x:c r="H498" s="11"/>
+      <x:c r="H498" s="11" t="str">
+        <x:v>(${final_summary_report_type} = 'gt' or ${final_summary_report_type} = 'horeca')</x:v>
+      </x:c>
       <x:c r="I498" s="11"/>
       <x:c r="J498" s="11"/>
       <x:c r="K498" s="11"/>
@@ -13782,7 +13876,7 @@
       </x:c>
       <x:c r="G505" s="11"/>
       <x:c r="H505" s="11" t="str">
-        <x:v>string-length(normalize-space(${final_summary_report_type})) = 0 or ${final_summary_report_type} = 'gt'</x:v>
+        <x:v>${final_summary_report_type} = 'gt'</x:v>
       </x:c>
       <x:c r="I505" s="11"/>
       <x:c r="J505" s="11"/>
@@ -14044,7 +14138,7 @@
       </x:c>
       <x:c r="G515" s="11"/>
       <x:c r="H515" s="11" t="str">
-        <x:v>string-length(normalize-space(${final_summary_report_type})) = 0 or ${final_summary_report_type} = 'gt'</x:v>
+        <x:v>${final_summary_report_type} = 'gt'</x:v>
       </x:c>
       <x:c r="I515" s="11"/>
       <x:c r="J515" s="11"/>
@@ -14225,7 +14319,7 @@
       </x:c>
       <x:c r="G522" s="11"/>
       <x:c r="H522" s="11" t="str">
-        <x:v>string-length(normalize-space(${final_summary_report_type})) = 0 or ${final_summary_report_type} = 'gt'</x:v>
+        <x:v>${final_summary_report_type} = 'gt'</x:v>
       </x:c>
       <x:c r="I522" s="11"/>
       <x:c r="J522" s="11"/>
@@ -14406,7 +14500,7 @@
       </x:c>
       <x:c r="G529" s="11"/>
       <x:c r="H529" s="11" t="str">
-        <x:v>string-length(normalize-space(${final_summary_report_type})) = 0 or ${final_summary_report_type} = 'gt'</x:v>
+        <x:v>${final_summary_report_type} = 'gt'</x:v>
       </x:c>
       <x:c r="I529" s="11"/>
       <x:c r="J529" s="11"/>
@@ -14587,7 +14681,7 @@
       </x:c>
       <x:c r="G536" s="11"/>
       <x:c r="H536" s="11" t="str">
-        <x:v>string-length(normalize-space(${final_summary_report_type})) = 0 or ${final_summary_report_type} = 'gt'</x:v>
+        <x:v>${final_summary_report_type} = 'gt'</x:v>
       </x:c>
       <x:c r="I536" s="11"/>
       <x:c r="J536" s="11"/>
@@ -14785,7 +14879,7 @@
       </x:c>
       <x:c r="G544" s="11"/>
       <x:c r="H544" s="11" t="str">
-        <x:v>not(normalize-space(${outlet_name}) = 'បូកសរុបរួម' or normalize-space(${outlet_name}) = 'បូកសរុបរូម' or normalize-space(${outlet_name}) = 'សរុបរួម' or normalize-space(${outlet_name}) = 'បួកសរុបរួម')</x:v>
+        <x:v>(${final_summary_report_type} = 'gt' or ${final_summary_report_type} = 'horeca') and (not(normalize-space(${outlet_name}) = 'បូកសរុបរួម' or normalize-space(${outlet_name}) = 'បូកសរុបរូម' or normalize-space(${outlet_name}) = 'សរុបរួម' or normalize-space(${outlet_name}) = 'បួកសរុបរួម'))</x:v>
       </x:c>
       <x:c r="I544" s="11"/>
       <x:c r="J544" s="11"/>
@@ -14905,7 +14999,9 @@
       <x:c r="E549" s="11"/>
       <x:c r="F549" s="11"/>
       <x:c r="G549" s="11"/>
-      <x:c r="H549" s="11"/>
+      <x:c r="H549" s="11" t="str">
+        <x:v>(${final_summary_report_type} = 'gt' or ${final_summary_report_type} = 'horeca')</x:v>
+      </x:c>
       <x:c r="I549" s="11"/>
       <x:c r="J549" s="11"/>
       <x:c r="K549" s="11"/>

</xml_diff>

<commit_message>
Remove CAMBODIA ED from HORECA form and report
</commit_message>
<xml_diff>
--- a/templates/KB_Market_Improvement_XLSForm_GT_HORECA.xlsx
+++ b/templates/KB_Market_Improvement_XLSForm_GT_HORECA.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="survey" sheetId="1" r:id="R656fd06bac004168"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="choices" sheetId="2" r:id="Re1688679d57a425a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="settings" sheetId="3" r:id="Rd6e944611b654d96"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bot_Logic" sheetId="4" r:id="R9595ba678a004b1d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bot_Data_Map" sheetId="5" r:id="R99663956829847bc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="survey" sheetId="1" r:id="Rcbad372994024d63"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="choices" sheetId="2" r:id="R359d423472f34e90"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="settings" sheetId="3" r:id="R809ec8351ba94169"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bot_Logic" sheetId="4" r:id="R8ebc5d4bb25948d2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bot_Data_Map" sheetId="5" r:id="Rac344dd6c54549ae"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -7253,7 +7253,7 @@
       </x:c>
       <x:c r="G250" s="11"/>
       <x:c r="H250" s="11" t="str">
-        <x:v>(${final_summary_report_type} = 'gt' or ${final_summary_report_type} = 'horeca')</x:v>
+        <x:v>${final_summary_report_type} = 'gt'</x:v>
       </x:c>
       <x:c r="I250" s="11"/>
       <x:c r="J250" s="11"/>

</xml_diff>